<commit_message>
Crear ejecutable ACTUALIZAR_CATALOGO.bat y sincronizar precio de Zakat World Cup a 270.000 desde Drive
</commit_message>
<xml_diff>
--- a/Catalogo_Perfumes_Ole_Diferente.xlsx
+++ b/Catalogo_Perfumes_Ole_Diferente.xlsx
@@ -28,40 +28,40 @@
     <t>Nombre</t>
   </si>
   <si>
+    <t>Precio ($ ARS)</t>
+  </si>
+  <si>
+    <t>Cant en stock</t>
+  </si>
+  <si>
     <t>1. MODIFICAR PRECIOS: Actualice directamente los valores numéricos en la columna 'Precio ($ ARS)'.</t>
   </si>
   <si>
-    <t>Precio ($ ARS)</t>
-  </si>
-  <si>
-    <t>Cant en stock</t>
+    <t>Por encargue</t>
+  </si>
+  <si>
+    <t>Categoría</t>
+  </si>
+  <si>
+    <t>Estado actual en Web</t>
+  </si>
+  <si>
+    <t>Notas / Observaciones</t>
   </si>
   <si>
     <t>2. CONTROL DE STOCK: En 'Cant en stock', coloque la cantidad de unidades físicas disponibles para entrega inmediata.</t>
   </si>
   <si>
-    <t>Por encargue</t>
-  </si>
-  <si>
-    <t>Categoría</t>
+    <t>9 AM Dive</t>
   </si>
   <si>
     <t>3. POR ENCARGUE: Escriba 'Sí' si el perfume se puede traer a pedido/seña, o 'No' si solo se vende de stock físico o no se trabaja.</t>
   </si>
   <si>
-    <t>Estado actual en Web</t>
-  </si>
-  <si>
-    <t>Notas / Observaciones</t>
-  </si>
-  <si>
     <t>4. AGREGAR PERFUMES NUEVOS: Puede agregar nuevas filas al final de la lista con su Nombre, Precio y Estado.</t>
   </si>
   <si>
     <t>5. SINCRONIZACIÓN AUTOMÁTICA: Guarde el archivo y envíelo; con solo ejecutar el script de sincronización, toda la tienda web y la base de datos se actualizarán al instante.</t>
-  </si>
-  <si>
-    <t>9 AM Dive</t>
   </si>
   <si>
     <t>Sí</t>
@@ -604,22 +604,22 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>5</v>
-      </c>
       <c r="E1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="H1" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2">
@@ -627,7 +627,7 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C2" s="2">
         <v>77500.0</v>
@@ -2395,8 +2395,8 @@
       <c r="B75" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C75" s="2">
-        <v>205000.0</v>
+      <c r="C75" s="5">
+        <v>270000.0</v>
       </c>
       <c r="D75" s="3">
         <v>0.0</v>
@@ -3356,27 +3356,27 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Actualizacion automatica de precios y stock desde Google Drive
</commit_message>
<xml_diff>
--- a/Catalogo_Perfumes_Ole_Diferente.xlsx
+++ b/Catalogo_Perfumes_Ole_Diferente.xlsx
@@ -19,24 +19,36 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="100">
   <si>
+    <t>GUÍA RÁPIDA DE USO</t>
+  </si>
+  <si>
     <t>N°</t>
   </si>
   <si>
-    <t>GUÍA RÁPIDA DE USO</t>
+    <t>1. MODIFICAR PRECIOS: Actualice directamente los valores numéricos en la columna 'Precio ($ ARS)'.</t>
+  </si>
+  <si>
+    <t>2. CONTROL DE STOCK: En 'Cant en stock', coloque la cantidad de unidades físicas disponibles para entrega inmediata.</t>
+  </si>
+  <si>
+    <t>3. POR ENCARGUE: Escriba 'Sí' si el perfume se puede traer a pedido/seña, o 'No' si solo se vende de stock físico o no se trabaja.</t>
+  </si>
+  <si>
+    <t>4. AGREGAR PERFUMES NUEVOS: Puede agregar nuevas filas al final de la lista con su Nombre, Precio y Estado.</t>
   </si>
   <si>
     <t>Nombre</t>
   </si>
   <si>
+    <t>5. SINCRONIZACIÓN AUTOMÁTICA: Guarde el archivo y envíelo; con solo ejecutar el script de sincronización, toda la tienda web y la base de datos se actualizarán al instante.</t>
+  </si>
+  <si>
     <t>Precio ($ ARS)</t>
   </si>
   <si>
     <t>Cant en stock</t>
   </si>
   <si>
-    <t>1. MODIFICAR PRECIOS: Actualice directamente los valores numéricos en la columna 'Precio ($ ARS)'.</t>
-  </si>
-  <si>
     <t>Por encargue</t>
   </si>
   <si>
@@ -49,19 +61,7 @@
     <t>Notas / Observaciones</t>
   </si>
   <si>
-    <t>2. CONTROL DE STOCK: En 'Cant en stock', coloque la cantidad de unidades físicas disponibles para entrega inmediata.</t>
-  </si>
-  <si>
     <t>9 AM Dive</t>
-  </si>
-  <si>
-    <t>3. POR ENCARGUE: Escriba 'Sí' si el perfume se puede traer a pedido/seña, o 'No' si solo se vende de stock físico o no se trabaja.</t>
-  </si>
-  <si>
-    <t>4. AGREGAR PERFUMES NUEVOS: Puede agregar nuevas filas al final de la lista con su Nombre, Precio y Estado.</t>
-  </si>
-  <si>
-    <t>5. SINCRONIZACIÓN AUTOMÁTICA: Guarde el archivo y envíelo; con solo ejecutar el script de sincronización, toda la tienda web y la base de datos se actualizarán al instante.</t>
   </si>
   <si>
     <t>Sí</t>
@@ -323,8 +323,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -358,20 +359,23 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="1" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="1" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="1" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -598,28 +602,28 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2">
@@ -627,7 +631,7 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C2" s="2">
         <v>77500.0</v>
@@ -721,8 +725,8 @@
       <c r="B6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="2">
-        <v>110000.0</v>
+      <c r="C6" s="4">
+        <v>125000.0</v>
       </c>
       <c r="D6" s="3">
         <v>0.0</v>
@@ -813,8 +817,8 @@
       <c r="B10" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="2">
-        <v>67000.0</v>
+      <c r="C10" s="4">
+        <v>78000.0</v>
       </c>
       <c r="D10" s="3">
         <v>0.0</v>
@@ -1859,8 +1863,8 @@
       <c r="B53" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C53" s="2">
-        <v>74000.0</v>
+      <c r="C53" s="4">
+        <v>84000.0</v>
       </c>
       <c r="D53" s="3">
         <v>1.0</v>
@@ -1957,27 +1961,27 @@
       <c r="A57" s="1">
         <v>55.0</v>
       </c>
-      <c r="B57" s="4" t="s">
+      <c r="B57" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="C57" s="5">
+      <c r="C57" s="4">
         <v>72000.0</v>
       </c>
       <c r="D57" s="6">
         <v>1.0</v>
       </c>
-      <c r="E57" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F57" s="4" t="s">
+      <c r="E57" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F57" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="G57" s="4" t="s">
+      <c r="G57" s="5" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="4">
+      <c r="A58" s="5">
         <v>56.0</v>
       </c>
       <c r="B58" s="1" t="s">
@@ -2003,7 +2007,7 @@
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
-      <c r="A59" s="4">
+      <c r="A59" s="5">
         <v>57.0</v>
       </c>
       <c r="B59" s="1" t="s">
@@ -2026,7 +2030,7 @@
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
-      <c r="A60" s="4">
+      <c r="A60" s="5">
         <v>58.0</v>
       </c>
       <c r="B60" s="1" t="s">
@@ -2049,7 +2053,7 @@
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
-      <c r="A61" s="4">
+      <c r="A61" s="5">
         <v>59.0</v>
       </c>
       <c r="B61" s="1" t="s">
@@ -2075,7 +2079,7 @@
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
-      <c r="A62" s="4">
+      <c r="A62" s="5">
         <v>60.0</v>
       </c>
       <c r="B62" s="1" t="s">
@@ -2101,7 +2105,7 @@
       </c>
     </row>
     <row r="63" ht="15.75" customHeight="1">
-      <c r="A63" s="4">
+      <c r="A63" s="5">
         <v>61.0</v>
       </c>
       <c r="B63" s="1" t="s">
@@ -2127,7 +2131,7 @@
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
-      <c r="A64" s="4">
+      <c r="A64" s="5">
         <v>62.0</v>
       </c>
       <c r="B64" s="1" t="s">
@@ -2150,7 +2154,7 @@
       </c>
     </row>
     <row r="65" ht="15.75" customHeight="1">
-      <c r="A65" s="4">
+      <c r="A65" s="5">
         <v>63.0</v>
       </c>
       <c r="B65" s="1" t="s">
@@ -2176,7 +2180,7 @@
       </c>
     </row>
     <row r="66" ht="15.75" customHeight="1">
-      <c r="A66" s="4">
+      <c r="A66" s="5">
         <v>64.0</v>
       </c>
       <c r="B66" s="1" t="s">
@@ -2202,7 +2206,7 @@
       </c>
     </row>
     <row r="67" ht="15.75" customHeight="1">
-      <c r="A67" s="4">
+      <c r="A67" s="5">
         <v>65.0</v>
       </c>
       <c r="B67" s="1" t="s">
@@ -2228,7 +2232,7 @@
       </c>
     </row>
     <row r="68" ht="15.75" customHeight="1">
-      <c r="A68" s="4">
+      <c r="A68" s="5">
         <v>66.0</v>
       </c>
       <c r="B68" s="1" t="s">
@@ -2251,7 +2255,7 @@
       </c>
     </row>
     <row r="69" ht="15.75" customHeight="1">
-      <c r="A69" s="4">
+      <c r="A69" s="5">
         <v>67.0</v>
       </c>
       <c r="B69" s="1" t="s">
@@ -2274,7 +2278,7 @@
       </c>
     </row>
     <row r="70" ht="15.75" customHeight="1">
-      <c r="A70" s="4">
+      <c r="A70" s="5">
         <v>68.0</v>
       </c>
       <c r="B70" s="1" t="s">
@@ -2297,7 +2301,7 @@
       </c>
     </row>
     <row r="71" ht="15.75" customHeight="1">
-      <c r="A71" s="4">
+      <c r="A71" s="5">
         <v>69.0</v>
       </c>
       <c r="B71" s="1" t="s">
@@ -2320,7 +2324,7 @@
       </c>
     </row>
     <row r="72" ht="15.75" customHeight="1">
-      <c r="A72" s="4">
+      <c r="A72" s="5">
         <v>70.0</v>
       </c>
       <c r="B72" s="1" t="s">
@@ -2343,7 +2347,7 @@
       </c>
     </row>
     <row r="73" ht="15.75" customHeight="1">
-      <c r="A73" s="4">
+      <c r="A73" s="5">
         <v>71.0</v>
       </c>
       <c r="B73" s="1" t="s">
@@ -2366,7 +2370,7 @@
       </c>
     </row>
     <row r="74" ht="15.75" customHeight="1">
-      <c r="A74" s="4">
+      <c r="A74" s="5">
         <v>72.0</v>
       </c>
       <c r="B74" s="1" t="s">
@@ -2389,13 +2393,13 @@
       </c>
     </row>
     <row r="75" ht="15.75" customHeight="1">
-      <c r="A75" s="4">
+      <c r="A75" s="5">
         <v>73.0</v>
       </c>
       <c r="B75" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C75" s="5">
+      <c r="C75" s="4">
         <v>270000.0</v>
       </c>
       <c r="D75" s="3">
@@ -2411,7 +2415,10 @@
         <v>17</v>
       </c>
     </row>
-    <row r="76" ht="15.75" customHeight="1"/>
+    <row r="76" ht="15.75" customHeight="1">
+      <c r="A76" s="5"/>
+      <c r="C76" s="7"/>
+    </row>
     <row r="77" ht="15.75" customHeight="1"/>
     <row r="78" ht="15.75" customHeight="1"/>
     <row r="79" ht="15.75" customHeight="1"/>
@@ -3351,32 +3358,32 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>